<commit_message>
Update resources and configuration assets
</commit_message>
<xml_diff>
--- a/config/excel/InitUnits.xlsx
+++ b/config/excel/InitUnits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyZiegler\github\ra2\config\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A7CB543-60A7-453E-BC8D-B4CABDE692F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F7563BC-616C-4950-8508-F30F34597B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="30885" windowHeight="16065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1305" yWindow="1920" windowWidth="30885" windowHeight="16065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConfInitUnits" sheetId="1" r:id="rId1"/>
@@ -194,11 +194,11 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>30,0,32</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>灰熊坦克</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>20,0,32</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1020,7 +1020,7 @@
         <v>31</v>
       </c>
       <c r="H16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1046,7 +1046,7 @@
         <v>31</v>
       </c>
       <c r="H17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1072,7 +1072,7 @@
         <v>31</v>
       </c>
       <c r="H18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1092,13 +1092,13 @@
         <v>0</v>
       </c>
       <c r="F19" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="H19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>